<commit_message>
Update Attendance_2026_10_27: Set Khaled Malas to OFF (Rest Day)
</commit_message>
<xml_diff>
--- a/Attendance_2026_10_27.xlsx
+++ b/Attendance_2026_10_27.xlsx
@@ -901,48 +901,48 @@
       </c>
     </row>
     <row r="8" ht="24" customHeight="1">
-      <c r="A8" s="15" t="n">
+      <c r="A8" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="16" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>Khaled Mohammad Mlas</t>
         </is>
       </c>
-      <c r="C8" s="17" t="n">
+      <c r="C8" s="4" t="n">
         <v>46322</v>
       </c>
-      <c r="D8" s="18" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E8" s="18" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F8" s="18" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G8" s="18" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H8" s="19" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H8" s="7" t="inlineStr">
         <is>
           <t>محمد خالد ملص</t>
         </is>
       </c>
-      <c r="I8" s="20" t="inlineStr">
-        <is>
-          <t>⏳ Awaiting Report</t>
-        </is>
-      </c>
-      <c r="J8" s="16" t="inlineStr">
+      <c r="I8" s="8" t="inlineStr">
+        <is>
+          <t>OFF (Rest Day)</t>
+        </is>
+      </c>
+      <c r="J8" s="3" t="inlineStr">
         <is>
           <t>FlyDubi</t>
         </is>

</xml_diff>

<commit_message>
Update Hanan 27 Oct as OFF and log 28 Oct shifts for team
</commit_message>
<xml_diff>
--- a/Attendance_2026_10_27.xlsx
+++ b/Attendance_2026_10_27.xlsx
@@ -721,48 +721,48 @@
       </c>
     </row>
     <row r="4" ht="24" customHeight="1">
-      <c r="A4" s="15" t="n">
+      <c r="A4" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="16" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>Hanan Tinawi</t>
         </is>
       </c>
-      <c r="C4" s="17" t="n">
+      <c r="C4" s="4" t="n">
         <v>46322</v>
       </c>
-      <c r="D4" s="18" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E4" s="18" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F4" s="18" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G4" s="18" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H4" s="19" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>حنان تيناوي</t>
         </is>
       </c>
-      <c r="I4" s="20" t="inlineStr">
-        <is>
-          <t>⏳ Awaiting Report</t>
-        </is>
-      </c>
-      <c r="J4" s="16" t="inlineStr">
+      <c r="I4" s="8" t="inlineStr">
+        <is>
+          <t>OFF (Rest Day)</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
         <is>
           <t>FlyDubi</t>
         </is>

</xml_diff>